<commit_message>
Add Desktop sample/screenshot guide; continue past DNS wait
Document exact Power BI Desktop steps for the AppSource .pbix and
1366x768 screenshots, refresh sample Excel howto text, and note that
we can proceed while datalund.no TLS propagation finishes.

Co-authored-by: JonasL <Prez0@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ganttChart/downloads/GanttSampleData.xlsx
+++ b/ganttChart/downloads/GanttSampleData.xlsx
@@ -423,7 +423,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -716,8 +716,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="A1:A10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
   </cols>
@@ -725,10 +725,11 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Power BI Desktop test data for the custom Gantt visual</t>
-        </is>
-      </c>
-    </row>
+          <t>Power BI Desktop test data for DataLund Gantt</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -739,14 +740,14 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2. Import GanttChart.pbiviz (Visualizations … → Import a visual from a file).</t>
+          <t>2. Import downloads/ganttChart.pbiviz (Visualizations … → Import a visual from a file).</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>3. Bind: Task→Task, Start Date→Start, End Date→End, Duration→Duration (optional extras: Progress, Group, Resource).</t>
+          <t>3. Bind: Task→Task, Start Date→Start, End Date→End, Duration→Duration; optional Progress, Group, Resource.</t>
         </is>
       </c>
     </row>
@@ -757,6 +758,16 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Full AppSource Desktop steps: ganttChart/docs/DESKTOP_SAMPLE.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rename download package to DataLundGantt.pbiviz
Use a branded download filename while keeping the internal visual name
and GUID unchanged. Update docs, sample Excel howto, and copy path.

Co-authored-by: JonasL <Prez0@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ganttChart/downloads/GanttSampleData.xlsx
+++ b/ganttChart/downloads/GanttSampleData.xlsx
@@ -716,7 +716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -729,7 +729,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -740,7 +739,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2. Import downloads/ganttChart.pbiviz (Visualizations … → Import a visual from a file).</t>
+          <t>2. Import downloads/DataLundGantt.pbiviz (Visualizations … → Import a visual from a file).</t>
         </is>
       </c>
     </row>
@@ -765,9 +764,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add DataLund Gantt Lab experimental visual
Separate GUID so Lab can coexist with the AppSource visual. Adds a
3/6/9/12M time-window toolbar, expand/collapse, predecessor dependency
arrows, status coloring, month grid, and richer bar/milestone/today
graphics. Documented as not for AppSource.

Co-authored-by: JonasL <Prez0@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ganttChart/downloads/GanttSampleData.xlsx
+++ b/ganttChart/downloads/GanttSampleData.xlsx
@@ -20,16 +20,13 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -52,11 +49,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -422,68 +417,64 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-  </cols>
+  <dimension ref="A1:H11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Task</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Start</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>End</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Duration</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Progress</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Group</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Resource</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Predecessor</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Requirements</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="n">
-        <v>46027</v>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>46036</v>
-      </c>
-      <c r="E2" s="3" t="n">
+          <t>Kickoff</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="n">
+        <v>46220</v>
+      </c>
+      <c r="C2" s="1" t="n">
+        <v>46220</v>
+      </c>
+      <c r="E2" t="n">
         <v>1</v>
       </c>
       <c r="F2" t="inlineStr">
@@ -500,17 +491,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Wireframes</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="n">
-        <v>46034</v>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>46043</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>0.85</v>
+          <t>Requirements</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="n">
+        <v>46222</v>
+      </c>
+      <c r="C3" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -519,50 +510,60 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Alex</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Kickoff</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>API Design</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="n">
-        <v>46037</v>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>46051</v>
-      </c>
-      <c r="E4" s="3" t="n">
-        <v>0.6</v>
+          <t>Wireframes</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>46230</v>
+      </c>
+      <c r="C4" s="1" t="n">
+        <v>46245</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.9</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Discovery</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Sam</t>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Requirements</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Frontend</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="n">
-        <v>46044</v>
-      </c>
-      <c r="C5" s="2" t="n">
-        <v>46065</v>
-      </c>
-      <c r="E5" s="3" t="n">
-        <v>0.35</v>
+          <t>API Design</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="n">
+        <v>46238</v>
+      </c>
+      <c r="C5" s="1" t="n">
+        <v>46258</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.55</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -571,24 +572,29 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Sam</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Requirements</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Backend</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="n">
-        <v>46044</v>
-      </c>
-      <c r="C6" s="2" t="n">
-        <v>46062</v>
-      </c>
-      <c r="E6" s="3" t="n">
-        <v>0.45</v>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="n">
+        <v>46245</v>
+      </c>
+      <c r="C6" s="1" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.35</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -597,24 +603,29 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Sam</t>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Wireframes</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Alpha Gate</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="n">
-        <v>46065</v>
-      </c>
-      <c r="C7" s="2" t="n">
-        <v>46065</v>
-      </c>
-      <c r="E7" s="3" t="n">
-        <v>1</v>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="n">
+        <v>46245</v>
+      </c>
+      <c r="C7" s="1" t="n">
+        <v>46275</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.4</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -623,50 +634,60 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Alex</t>
+          <t>Sam</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>API Design</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>QA</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="n">
-        <v>46062</v>
-      </c>
-      <c r="D8" t="n">
-        <v>14</v>
-      </c>
-      <c r="E8" s="3" t="n">
-        <v>0.1</v>
+          <t>Alpha Gate</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="n">
+        <v>46280</v>
+      </c>
+      <c r="C8" s="1" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Launch</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Riley</t>
+          <t>Alex</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Frontend</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>UAT</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="n">
-        <v>46072</v>
-      </c>
-      <c r="C9" s="2" t="n">
-        <v>46079</v>
-      </c>
-      <c r="E9" s="3" t="n">
-        <v>0</v>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="n">
+        <v>46270</v>
+      </c>
+      <c r="D9" t="n">
+        <v>21</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.15</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -675,33 +696,74 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Alex</t>
+          <t>Riley</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Backend</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>UAT</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="n">
+        <v>46285</v>
+      </c>
+      <c r="C10" s="1" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Launch</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Alex</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>Go-Live</t>
         </is>
       </c>
-      <c r="B10" s="2" t="n">
-        <v>46082</v>
-      </c>
-      <c r="C10" s="2" t="n">
-        <v>46082</v>
-      </c>
-      <c r="E10" s="3" t="n">
+      <c r="B11" s="1" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C11" s="1" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E11" t="n">
         <v>0</v>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>Launch</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>Alex</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>UAT</t>
         </is>
       </c>
     </row>
@@ -716,44 +778,48 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
-  <cols>
-    <col width="110" customWidth="1" min="1" max="1"/>
-  </cols>
+  <dimension ref="A1:A7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Power BI Desktop test data for the custom Gantt visual</t>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>DataLund Gantt Lab — experimental sample</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1. Home → Get data → Excel workbook → select this file → load Tasks.</t>
+          <t>1. Import downloads/DataLundGanttLab.pbiviz</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2. Import GanttChart.pbiviz (Visualizations … → Import a visual from a file).</t>
+          <t>2. Load Tasks sheet; bind Task, Start, End/Duration, Progress, Group, Resource, Predecessor</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>3. Bind: Task→Task, Start Date→Start, End Date→End, Duration→Duration (optional extras: Progress, Group, Resource).</t>
+          <t>3. Use toolbar 3M/6M/9M/12M/All — windows are centered on today</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Alpha Gate and Go-Live are zero-duration milestones. QA uses Duration instead of End.</t>
+          <t>4. Predecessor = upstream Task name (finish-to-start arrows)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>NOT for AppSource. See docs/EXPERIMENTAL.md</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Lab: optional planned vs actual baseline bars
Add Planned Start / Planned End wells and thinner baseline bars under
actual schedule bars. Core remains Task + Start + End; baselines and
all other wells stay optional. Format → Lab → Show planned bars.

Co-authored-by: JonasL <Prez0@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ganttChart/downloads/GanttSampleData.xlsx
+++ b/ganttChart/downloads/GanttSampleData.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -438,25 +438,35 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>PlannedStart</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>PlannedEnd</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>Duration</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Progress</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Group</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Resource</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Predecessor</t>
         </is>
@@ -474,15 +484,21 @@
       <c r="C2" s="1" t="n">
         <v>46220</v>
       </c>
-      <c r="E2" t="n">
+      <c r="D2" s="1" t="n">
+        <v>46218</v>
+      </c>
+      <c r="E2" s="1" t="n">
+        <v>46218</v>
+      </c>
+      <c r="G2" t="n">
         <v>1</v>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Discovery</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>Alex</t>
         </is>
@@ -500,20 +516,26 @@
       <c r="C3" s="1" t="n">
         <v>46235</v>
       </c>
-      <c r="E3" t="n">
+      <c r="D3" s="1" t="n">
+        <v>46220</v>
+      </c>
+      <c r="E3" s="1" t="n">
+        <v>46232</v>
+      </c>
+      <c r="G3" t="n">
         <v>1</v>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>Discovery</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>Alex</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Kickoff</t>
         </is>
@@ -531,20 +553,26 @@
       <c r="C4" s="1" t="n">
         <v>46245</v>
       </c>
-      <c r="E4" t="n">
+      <c r="D4" s="1" t="n">
+        <v>46228</v>
+      </c>
+      <c r="E4" s="1" t="n">
+        <v>46240</v>
+      </c>
+      <c r="G4" t="n">
         <v>0.9</v>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>Discovery</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>Jordan</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>Requirements</t>
         </is>
@@ -562,20 +590,26 @@
       <c r="C5" s="1" t="n">
         <v>46258</v>
       </c>
-      <c r="E5" t="n">
+      <c r="D5" s="1" t="n">
+        <v>46236</v>
+      </c>
+      <c r="E5" s="1" t="n">
+        <v>46252</v>
+      </c>
+      <c r="G5" t="n">
         <v>0.55</v>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>Build</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>Sam</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>Requirements</t>
         </is>
@@ -593,20 +627,26 @@
       <c r="C6" s="1" t="n">
         <v>46280</v>
       </c>
-      <c r="E6" t="n">
+      <c r="D6" s="1" t="n">
+        <v>46242</v>
+      </c>
+      <c r="E6" s="1" t="n">
+        <v>46272</v>
+      </c>
+      <c r="G6" t="n">
         <v>0.35</v>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>Build</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>Jordan</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>Wireframes</t>
         </is>
@@ -624,20 +664,26 @@
       <c r="C7" s="1" t="n">
         <v>46275</v>
       </c>
-      <c r="E7" t="n">
+      <c r="D7" s="1" t="n">
+        <v>46242</v>
+      </c>
+      <c r="E7" s="1" t="n">
+        <v>46268</v>
+      </c>
+      <c r="G7" t="n">
         <v>0.4</v>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>Build</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>Sam</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>API Design</t>
         </is>
@@ -655,20 +701,26 @@
       <c r="C8" s="1" t="n">
         <v>46280</v>
       </c>
-      <c r="E8" t="n">
+      <c r="D8" s="1" t="n">
+        <v>46272</v>
+      </c>
+      <c r="E8" s="1" t="n">
+        <v>46272</v>
+      </c>
+      <c r="G8" t="n">
         <v>0</v>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>Build</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>Alex</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>Frontend</t>
         </is>
@@ -683,23 +735,29 @@
       <c r="B9" s="1" t="n">
         <v>46270</v>
       </c>
-      <c r="D9" t="n">
+      <c r="D9" s="1" t="n">
+        <v>46265</v>
+      </c>
+      <c r="E9" s="1" t="n">
+        <v>46285</v>
+      </c>
+      <c r="F9" t="n">
         <v>21</v>
       </c>
-      <c r="E9" t="n">
+      <c r="G9" t="n">
         <v>0.15</v>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>Launch</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>Riley</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>Backend</t>
         </is>
@@ -717,20 +775,26 @@
       <c r="C10" s="1" t="n">
         <v>46295</v>
       </c>
-      <c r="E10" t="n">
+      <c r="D10" s="1" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E10" s="1" t="n">
+        <v>46290</v>
+      </c>
+      <c r="G10" t="n">
         <v>0</v>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>Launch</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>Alex</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>QA</t>
         </is>
@@ -748,20 +812,26 @@
       <c r="C11" s="1" t="n">
         <v>46300</v>
       </c>
-      <c r="E11" t="n">
+      <c r="D11" s="1" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E11" s="1" t="n">
+        <v>46292</v>
+      </c>
+      <c r="G11" t="n">
         <v>0</v>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>Launch</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>Alex</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>UAT</t>
         </is>
@@ -778,7 +848,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -791,33 +861,40 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1. Import downloads/DataLundGanttLab.pbiviz</t>
+          <t>Required: Task + Start + End (or Duration). Everything else is optional.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2. Load Tasks sheet; bind Task, Start, End/Duration, Progress, Group, Resource, Predecessor</t>
+          <t>1. Import downloads/DataLundGanttLab.pbiviz</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>3. Use toolbar 3M/6M/9M/12M/All — windows are centered on today</t>
+          <t>2. Bind Start/End as actual; PlannedStart/PlannedEnd as baseline (optional)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>4. Predecessor = upstream Task name (finish-to-start arrows)</t>
+          <t>3. Format → Lab → Show planned bars (on by default when data present)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
+        <is>
+          <t>4. Progress is optional and off by default in Format → Lab</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>NOT for AppSource. See docs/EXPERIMENTAL.md</t>
         </is>

</xml_diff>

<commit_message>
Fix sample Excel dates for Power BI type detection
Use Excel built-in date format (numFmtId 14) and an Excel Table so
Start/End/Planned* import as Date instead of Whole Number.

Co-authored-by: JonasL <Prez0@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ganttChart/downloads/GanttSampleData.xlsx
+++ b/ganttChart/downloads/GanttSampleData.xlsx
@@ -18,15 +18,22 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="2">
@@ -49,9 +56,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -126,6 +136,25 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tasks" displayName="Tasks" ref="A1:J11" headerRowCount="1">
+  <autoFilter ref="A1:J11"/>
+  <tableColumns count="10">
+    <tableColumn id="1" name="Task"/>
+    <tableColumn id="2" name="Start"/>
+    <tableColumn id="3" name="End"/>
+    <tableColumn id="4" name="PlannedStart"/>
+    <tableColumn id="5" name="PlannedEnd"/>
+    <tableColumn id="6" name="Duration"/>
+    <tableColumn id="7" name="Progress"/>
+    <tableColumn id="8" name="Group"/>
+    <tableColumn id="9" name="Resource"/>
+    <tableColumn id="10" name="Predecessor"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -419,54 +448,66 @@
   </sheetPr>
   <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Task</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Start</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>End</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>PlannedStart</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>PlannedEnd</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Duration</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Progress</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Group</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Resource</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Predecessor</t>
         </is>
@@ -478,19 +519,19 @@
           <t>Kickoff</t>
         </is>
       </c>
-      <c r="B2" s="1" t="n">
+      <c r="B2" s="2" t="n">
         <v>46220</v>
       </c>
-      <c r="C2" s="1" t="n">
+      <c r="C2" s="2" t="n">
         <v>46220</v>
       </c>
-      <c r="D2" s="1" t="n">
+      <c r="D2" s="2" t="n">
         <v>46218</v>
       </c>
-      <c r="E2" s="1" t="n">
+      <c r="E2" s="2" t="n">
         <v>46218</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2" s="3" t="n">
         <v>1</v>
       </c>
       <c r="H2" t="inlineStr">
@@ -510,19 +551,19 @@
           <t>Requirements</t>
         </is>
       </c>
-      <c r="B3" s="1" t="n">
+      <c r="B3" s="2" t="n">
         <v>46222</v>
       </c>
-      <c r="C3" s="1" t="n">
+      <c r="C3" s="2" t="n">
         <v>46235</v>
       </c>
-      <c r="D3" s="1" t="n">
+      <c r="D3" s="2" t="n">
         <v>46220</v>
       </c>
-      <c r="E3" s="1" t="n">
+      <c r="E3" s="2" t="n">
         <v>46232</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3" s="3" t="n">
         <v>1</v>
       </c>
       <c r="H3" t="inlineStr">
@@ -547,19 +588,19 @@
           <t>Wireframes</t>
         </is>
       </c>
-      <c r="B4" s="1" t="n">
+      <c r="B4" s="2" t="n">
         <v>46230</v>
       </c>
-      <c r="C4" s="1" t="n">
+      <c r="C4" s="2" t="n">
         <v>46245</v>
       </c>
-      <c r="D4" s="1" t="n">
+      <c r="D4" s="2" t="n">
         <v>46228</v>
       </c>
-      <c r="E4" s="1" t="n">
+      <c r="E4" s="2" t="n">
         <v>46240</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4" s="3" t="n">
         <v>0.9</v>
       </c>
       <c r="H4" t="inlineStr">
@@ -584,19 +625,19 @@
           <t>API Design</t>
         </is>
       </c>
-      <c r="B5" s="1" t="n">
+      <c r="B5" s="2" t="n">
         <v>46238</v>
       </c>
-      <c r="C5" s="1" t="n">
+      <c r="C5" s="2" t="n">
         <v>46258</v>
       </c>
-      <c r="D5" s="1" t="n">
+      <c r="D5" s="2" t="n">
         <v>46236</v>
       </c>
-      <c r="E5" s="1" t="n">
+      <c r="E5" s="2" t="n">
         <v>46252</v>
       </c>
-      <c r="G5" t="n">
+      <c r="G5" s="3" t="n">
         <v>0.55</v>
       </c>
       <c r="H5" t="inlineStr">
@@ -621,19 +662,19 @@
           <t>Frontend</t>
         </is>
       </c>
-      <c r="B6" s="1" t="n">
+      <c r="B6" s="2" t="n">
         <v>46245</v>
       </c>
-      <c r="C6" s="1" t="n">
+      <c r="C6" s="2" t="n">
         <v>46280</v>
       </c>
-      <c r="D6" s="1" t="n">
+      <c r="D6" s="2" t="n">
         <v>46242</v>
       </c>
-      <c r="E6" s="1" t="n">
+      <c r="E6" s="2" t="n">
         <v>46272</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G6" s="3" t="n">
         <v>0.35</v>
       </c>
       <c r="H6" t="inlineStr">
@@ -658,19 +699,19 @@
           <t>Backend</t>
         </is>
       </c>
-      <c r="B7" s="1" t="n">
+      <c r="B7" s="2" t="n">
         <v>46245</v>
       </c>
-      <c r="C7" s="1" t="n">
+      <c r="C7" s="2" t="n">
         <v>46275</v>
       </c>
-      <c r="D7" s="1" t="n">
+      <c r="D7" s="2" t="n">
         <v>46242</v>
       </c>
-      <c r="E7" s="1" t="n">
+      <c r="E7" s="2" t="n">
         <v>46268</v>
       </c>
-      <c r="G7" t="n">
+      <c r="G7" s="3" t="n">
         <v>0.4</v>
       </c>
       <c r="H7" t="inlineStr">
@@ -695,19 +736,19 @@
           <t>Alpha Gate</t>
         </is>
       </c>
-      <c r="B8" s="1" t="n">
+      <c r="B8" s="2" t="n">
         <v>46280</v>
       </c>
-      <c r="C8" s="1" t="n">
+      <c r="C8" s="2" t="n">
         <v>46280</v>
       </c>
-      <c r="D8" s="1" t="n">
+      <c r="D8" s="2" t="n">
         <v>46272</v>
       </c>
-      <c r="E8" s="1" t="n">
+      <c r="E8" s="2" t="n">
         <v>46272</v>
       </c>
-      <c r="G8" t="n">
+      <c r="G8" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H8" t="inlineStr">
@@ -732,19 +773,19 @@
           <t>QA</t>
         </is>
       </c>
-      <c r="B9" s="1" t="n">
+      <c r="B9" s="2" t="n">
         <v>46270</v>
       </c>
-      <c r="D9" s="1" t="n">
+      <c r="D9" s="2" t="n">
         <v>46265</v>
       </c>
-      <c r="E9" s="1" t="n">
+      <c r="E9" s="2" t="n">
         <v>46285</v>
       </c>
       <c r="F9" t="n">
         <v>21</v>
       </c>
-      <c r="G9" t="n">
+      <c r="G9" s="3" t="n">
         <v>0.15</v>
       </c>
       <c r="H9" t="inlineStr">
@@ -769,19 +810,19 @@
           <t>UAT</t>
         </is>
       </c>
-      <c r="B10" s="1" t="n">
+      <c r="B10" s="2" t="n">
         <v>46285</v>
       </c>
-      <c r="C10" s="1" t="n">
+      <c r="C10" s="2" t="n">
         <v>46295</v>
       </c>
-      <c r="D10" s="1" t="n">
+      <c r="D10" s="2" t="n">
         <v>46280</v>
       </c>
-      <c r="E10" s="1" t="n">
+      <c r="E10" s="2" t="n">
         <v>46290</v>
       </c>
-      <c r="G10" t="n">
+      <c r="G10" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H10" t="inlineStr">
@@ -806,19 +847,19 @@
           <t>Go-Live</t>
         </is>
       </c>
-      <c r="B11" s="1" t="n">
+      <c r="B11" s="2" t="n">
         <v>46300</v>
       </c>
-      <c r="C11" s="1" t="n">
+      <c r="C11" s="2" t="n">
         <v>46300</v>
       </c>
-      <c r="D11" s="1" t="n">
+      <c r="D11" s="2" t="n">
         <v>46292</v>
       </c>
-      <c r="E11" s="1" t="n">
+      <c r="E11" s="2" t="n">
         <v>46292</v>
       </c>
-      <c r="G11" t="n">
+      <c r="G11" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H11" t="inlineStr">
@@ -839,6 +880,9 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -850,11 +894,14 @@
   </sheetPr>
   <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="92" customWidth="1" min="1" max="1"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>DataLund Gantt Lab — experimental sample</t>
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>DataLund Gantt Lab — sample data</t>
         </is>
       </c>
     </row>
@@ -868,35 +915,35 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1. Import downloads/DataLundGanttLab.pbiviz</t>
+          <t>Date columns use Excel date format so Power BI should detect them as Date (not Whole Number).</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2. Bind Start/End as actual; PlannedStart/PlannedEnd as baseline (optional)</t>
+          <t>1. Get data → Excel → load sheet Tasks (or table Tasks).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>3. Format → Lab → Show planned bars (on by default when data present)</t>
+          <t>2. If a date column still shows numbers: Transform → Data type → Date.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>4. Progress is optional and off by default in Format → Lab</t>
+          <t>3. Import DataLundGanttLab.pbiviz and bind fields (Start/End = actual; Planned* = baseline).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>NOT for AppSource. See docs/EXPERIMENTAL.md</t>
+          <t>4. Format → Lab: Show planned bars on; Show progress off unless you want fills.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Lab: realistic sample data + clearer planned envelope
Rewrite sample slips to 0–5 days so planned and actual overlap
readably. Draw planned as a taller outline envelope behind actual
instead of a thin stub that disappears under the bar.

Co-authored-by: JonasL <Prez0@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ganttChart/downloads/GanttSampleData.xlsx
+++ b/ganttChart/downloads/GanttSampleData.xlsx
@@ -56,11 +56,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -153,7 +152,7 @@
     <tableColumn id="9" name="Resource"/>
     <tableColumn id="10" name="Predecessor"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
 </file>
 
@@ -520,19 +519,16 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46220</v>
+        <v>46219</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>46220</v>
+        <v>46219</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>46218</v>
-      </c>
-      <c r="G2" s="3" t="n">
-        <v>1</v>
+        <v>46219</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -555,7 +551,7 @@
         <v>46222</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>46235</v>
+        <v>46234</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>46220</v>
@@ -563,9 +559,6 @@
       <c r="E3" s="2" t="n">
         <v>46232</v>
       </c>
-      <c r="G3" s="3" t="n">
-        <v>1</v>
-      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>Discovery</t>
@@ -592,16 +585,13 @@
         <v>46230</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>46245</v>
+        <v>46242</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>46228</v>
+        <v>46230</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>46240</v>
-      </c>
-      <c r="G4" s="3" t="n">
-        <v>0.9</v>
+        <v>46242</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -626,10 +616,10 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>46258</v>
+        <v>46256</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>46236</v>
@@ -637,9 +627,6 @@
       <c r="E5" s="2" t="n">
         <v>46252</v>
       </c>
-      <c r="G5" s="3" t="n">
-        <v>0.55</v>
-      </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>Build</t>
@@ -666,17 +653,14 @@
         <v>46245</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>46280</v>
+        <v>46272</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="E6" s="2" t="n">
         <v>46272</v>
       </c>
-      <c r="G6" s="3" t="n">
-        <v>0.35</v>
-      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>Build</t>
@@ -703,16 +687,13 @@
         <v>46245</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>46275</v>
+        <v>46270</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>46242</v>
+        <v>46245</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>46268</v>
-      </c>
-      <c r="G7" s="3" t="n">
-        <v>0.4</v>
+        <v>46267</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -737,19 +718,16 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>46280</v>
+        <v>46275</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>46280</v>
+        <v>46275</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>46272</v>
+        <v>46270</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>46272</v>
-      </c>
-      <c r="G8" s="3" t="n">
-        <v>0</v>
+        <v>46270</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -774,19 +752,16 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>46270</v>
+        <v>46268</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="F9" t="n">
-        <v>21</v>
-      </c>
-      <c r="G9" s="3" t="n">
-        <v>0.15</v>
+        <v>18</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -811,19 +786,16 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>46285</v>
+        <v>46284</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>46295</v>
+        <v>46293</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>46280</v>
+        <v>46282</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>46290</v>
-      </c>
-      <c r="G10" s="3" t="n">
-        <v>0</v>
+        <v>46291</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -848,19 +820,16 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>46300</v>
+        <v>46298</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>46300</v>
+        <v>46298</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>46292</v>
+        <v>46294</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>46292</v>
-      </c>
-      <c r="G11" s="3" t="n">
-        <v>0</v>
+        <v>46294</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -892,14 +861,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="92" customWidth="1" min="1" max="1"/>
+    <col width="96" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>DataLund Gantt Lab — sample data</t>
         </is>
@@ -915,35 +884,49 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Date columns use Excel date format so Power BI should detect them as Date (not Whole Number).</t>
+          <t>PlannedStart/PlannedEnd = baseline. Sample uses small slips (0–5 days) so both planned and actual stay readable.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1. Get data → Excel → load sheet Tasks (or table Tasks).</t>
+          <t>Progress is blank on purpose — leave Progress unbound, or keep Format → Lab → Show progress off.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2. If a date column still shows numbers: Transform → Data type → Date.</t>
+          <t>1. Get data → Excel → load table Tasks. Confirm Start/End/Planned* are Date type.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>3. Import DataLundGanttLab.pbiviz and bind fields (Start/End = actual; Planned* = baseline).</t>
+          <t>2. Import DataLundGanttLab.pbiviz.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>4. Format → Lab: Show planned bars on; Show progress off unless you want fills.</t>
+          <t>3. Bind: Task, Start→Start Date, End→End Date, PlannedStart, PlannedEnd, Group, Resource, Predecessor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>4. Do not bind Progress unless you want fills. Duration only needed for QA in this file.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>5. Try toolbar 6M (default-friendly). Colors = status (late / on track / future), not group.</t>
         </is>
       </c>
     </row>

</xml_diff>